<commit_message>
Refresh business report sample uploads
</commit_message>
<xml_diff>
--- a/sample_uploads/content.xlsx
+++ b/sample_uploads/content.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Trend" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Health" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Metrics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Revenue" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Forecast" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Health" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +42,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00014986"/>
+        <fgColor rgb="000F2038"/>
       </patternFill>
     </fill>
   </fills>
@@ -150,21 +151,22 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Revenue Trend by Segment</a:t>
+              <a:t>Q1 vs Q2 KPI Snapshot</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Revenue Trend'!B1</f>
+              <f>'KPI Summary'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -172,22 +174,14 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
-              <f>'Revenue Trend'!$A$2:$A$6</f>
+              <f>'KPI Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Revenue Trend'!$B$2:$B$6</f>
+              <f>'KPI Summary'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -196,7 +190,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Revenue Trend'!C1</f>
+              <f>'KPI Summary'!C1</f>
             </strRef>
           </tx>
           <spPr>
@@ -204,81 +198,27 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
-              <f>'Revenue Trend'!$A$2:$A$6</f>
+              <f>'KPI Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Revenue Trend'!$C$2:$C$6</f>
+              <f>'KPI Summary'!$C$2:$C$6</f>
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'Revenue Trend'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Revenue Trend'!$A$2:$A$6</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Revenue Trend'!$D$2:$D$6</f>
-            </numRef>
-          </val>
-        </ser>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
-      </lineChart>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Quarter</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -300,7 +240,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Revenue (M USD)</a:t>
+                  <a:t>Value</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -332,22 +272,21 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Weighted Pipeline by Stage</a:t>
+              <a:t>Monthly Revenue Trend</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
+      <lineChart>
+        <grouping val="standard"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Pipeline Health'!C1</f>
+              <f>'Monthly Revenue'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -355,42 +294,130 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
           <cat>
             <numRef>
-              <f>'Pipeline Health'!$A$2:$A$6</f>
+              <f>'Monthly Revenue'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Pipeline Health'!$C$2:$C$6</f>
+              <f>'Monthly Revenue'!$B$2:$B$7</f>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Revenue'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monthly Revenue'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Revenue'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Revenue'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monthly Revenue'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Revenue'!$D$2:$D$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Monthly Revenue'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monthly Revenue'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monthly Revenue'!$E$2:$E$7</f>
+            </numRef>
+          </val>
+        </ser>
         <axId val="10"/>
         <axId val="100"/>
-      </barChart>
+      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Stage</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -412,7 +439,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Pipeline (M USD)</a:t>
+                  <a:t>$M</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -436,12 +463,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>6</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5040000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -463,12 +490,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>6</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2700000"/>
+    <ext cx="5040000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -775,115 +802,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Quarter</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Enterprise ARR</t>
+          <t>Q1 Baseline</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>SMB ARR</t>
+          <t>Q2 Actual</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Services Revenue</t>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Target</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Q2 FY25</t>
+          <t>Revenue ($M)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>9.800000000000001</v>
+        <v>12.4</v>
       </c>
       <c r="C2" t="n">
-        <v>2.4</v>
+        <v>15.8</v>
       </c>
       <c r="D2" t="n">
-        <v>2.1</v>
+        <v>3.4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q3 FY25</t>
+          <t>Gross Margin (%)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.7</v>
+        <v>64</v>
       </c>
       <c r="C3" t="n">
-        <v>2.6</v>
+        <v>72</v>
       </c>
       <c r="D3" t="n">
-        <v>2.2</v>
+        <v>8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q4 FY25</t>
+          <t>NRR (%)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12.1</v>
+        <v>111</v>
       </c>
       <c r="C4" t="n">
-        <v>2.8</v>
+        <v>118</v>
       </c>
       <c r="D4" t="n">
-        <v>2.3</v>
+        <v>7</v>
+      </c>
+      <c r="E4" t="n">
+        <v>115</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q1 FY26</t>
+          <t>Pipeline Coverage (x)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14.4</v>
+        <v>2.8</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="D5" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q2 FY26 Forecast</t>
+          <t>SMB Churn (%)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16.2</v>
+        <v>3.1</v>
       </c>
       <c r="C6" t="n">
-        <v>3.3</v>
+        <v>2.4</v>
       </c>
       <c r="D6" t="n">
-        <v>2.7</v>
+        <v>-0.7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -898,94 +946,155 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Opportunities</t>
+          <t>Revenue $M</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Weighted Pipeline</t>
+          <t>Enterprise $M</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mid-market $M</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SMB $M</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Discovery</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>38</v>
+        <v>3.9</v>
       </c>
       <c r="C2" t="n">
-        <v>5.8</v>
+        <v>2.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Solution Fit</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>4.1</v>
       </c>
       <c r="C3" t="n">
-        <v>7.2</v>
+        <v>2.2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Business Case</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>14</v>
+        <v>4.4</v>
       </c>
       <c r="C4" t="n">
-        <v>8.6</v>
+        <v>2.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>4.8</v>
       </c>
       <c r="C5" t="n">
-        <v>6.9</v>
+        <v>2.7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Commit</t>
+          <t>May</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
       <c r="C6" t="n">
-        <v>4.4</v>
+        <v>3.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>
@@ -1000,115 +1109,231 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Segment</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Q4 Actual</t>
+          <t>Qualified Pipeline $M</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Q1 Actual</t>
+          <t>Stage 3 Conversion %</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Q2 Target</t>
+          <t>Q3 Base Forecast $M</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Q3 Upside $M</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Active Enterprise Accounts</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C2" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>10.1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>11.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Weekly Active Users</t>
+          <t>Mid-market</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18400</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>23500</v>
+        <v>31</v>
       </c>
       <c r="D3" t="n">
-        <v>29000</v>
+        <v>4.6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Expansion Pipeline</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>8.699999999999999</v>
+        <v>18</v>
       </c>
       <c r="D4" t="n">
-        <v>10.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>At-Risk ARR</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.1</v>
+        <v>57</v>
       </c>
       <c r="C5" t="n">
-        <v>1.6</v>
+        <v>33</v>
       </c>
       <c r="D5" t="n">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Median API Latency</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>410</v>
-      </c>
-      <c r="C6" t="n">
-        <v>332</v>
-      </c>
-      <c r="D6" t="n">
-        <v>300</v>
+        <v>17.2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>18.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Accounts &gt; $250K ARR</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Enterprise expansion momentum</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Gross Logo Retention %</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>91</v>
+      </c>
+      <c r="C3" t="n">
+        <v>94</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Improved onboarding and support response</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Median Activation Days</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SMB onboarding redesign impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>At-risk Enterprise Accounts</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Executive sponsor program reduced risk</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>